<commit_message>
Added notification according to language
</commit_message>
<xml_diff>
--- a/quickkart/data/catalog.xlsx
+++ b/quickkart/data/catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arnavshah/Desktop/BB-updated/quickkart/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D347DD9-F171-064D-87C3-809378F2BC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E339D5-0CDA-F141-83F4-D3E395E80542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15880" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dairy" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5533" uniqueCount="2154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5764" uniqueCount="2154">
   <si>
     <t>sku</t>
   </si>
@@ -9596,7 +9596,9 @@
     <col min="6" max="6" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="142.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9659,6 +9661,9 @@
       <c r="F2" s="2">
         <v>1</v>
       </c>
+      <c r="G2" t="s">
+        <v>155</v>
+      </c>
       <c r="H2" s="2">
         <v>25</v>
       </c>
@@ -9670,6 +9675,12 @@
       </c>
       <c r="K2" t="s">
         <v>16</v>
+      </c>
+      <c r="L2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M2" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9691,6 +9702,9 @@
       <c r="F3" s="2">
         <v>2</v>
       </c>
+      <c r="G3" t="s">
+        <v>155</v>
+      </c>
       <c r="H3" s="2">
         <v>50</v>
       </c>
@@ -9702,6 +9716,12 @@
       </c>
       <c r="K3" t="s">
         <v>16</v>
+      </c>
+      <c r="L3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9723,6 +9743,9 @@
       <c r="F4" s="2">
         <v>3</v>
       </c>
+      <c r="G4" t="s">
+        <v>155</v>
+      </c>
       <c r="H4" s="2">
         <v>40</v>
       </c>
@@ -9734,6 +9757,12 @@
       </c>
       <c r="K4" t="s">
         <v>16</v>
+      </c>
+      <c r="L4" t="s">
+        <v>155</v>
+      </c>
+      <c r="M4" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9755,6 +9784,9 @@
       <c r="F5" s="2">
         <v>4</v>
       </c>
+      <c r="G5" t="s">
+        <v>155</v>
+      </c>
       <c r="H5" s="2">
         <v>55</v>
       </c>
@@ -9766,6 +9798,12 @@
       </c>
       <c r="K5" t="s">
         <v>32</v>
+      </c>
+      <c r="L5" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9787,6 +9825,9 @@
       <c r="F6" s="2">
         <v>5</v>
       </c>
+      <c r="G6" t="s">
+        <v>155</v>
+      </c>
       <c r="H6" s="2">
         <v>60</v>
       </c>
@@ -9798,6 +9839,12 @@
       </c>
       <c r="K6" t="s">
         <v>32</v>
+      </c>
+      <c r="L6" t="s">
+        <v>155</v>
+      </c>
+      <c r="M6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9819,6 +9866,9 @@
       <c r="F7" s="2">
         <v>6</v>
       </c>
+      <c r="G7" t="s">
+        <v>155</v>
+      </c>
       <c r="H7" s="2">
         <v>45</v>
       </c>
@@ -9830,6 +9880,12 @@
       </c>
       <c r="K7" t="s">
         <v>32</v>
+      </c>
+      <c r="L7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M7" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9851,6 +9907,9 @@
       <c r="F8" s="2">
         <v>7</v>
       </c>
+      <c r="G8" t="s">
+        <v>155</v>
+      </c>
       <c r="H8" s="2">
         <v>80</v>
       </c>
@@ -9862,6 +9921,12 @@
       </c>
       <c r="K8" t="s">
         <v>48</v>
+      </c>
+      <c r="L8" t="s">
+        <v>155</v>
+      </c>
+      <c r="M8" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9883,6 +9948,9 @@
       <c r="F9" s="2">
         <v>8</v>
       </c>
+      <c r="G9" t="s">
+        <v>155</v>
+      </c>
       <c r="H9" s="2">
         <v>100</v>
       </c>
@@ -9894,6 +9962,12 @@
       </c>
       <c r="K9" t="s">
         <v>48</v>
+      </c>
+      <c r="L9" t="s">
+        <v>155</v>
+      </c>
+      <c r="M9" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9915,6 +9989,9 @@
       <c r="F10" s="2">
         <v>9</v>
       </c>
+      <c r="G10" t="s">
+        <v>155</v>
+      </c>
       <c r="H10" s="2">
         <v>20</v>
       </c>
@@ -9926,6 +10003,12 @@
       </c>
       <c r="K10" t="s">
         <v>48</v>
+      </c>
+      <c r="L10" t="s">
+        <v>155</v>
+      </c>
+      <c r="M10" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9947,6 +10030,9 @@
       <c r="F11" s="2">
         <v>10</v>
       </c>
+      <c r="G11" t="s">
+        <v>155</v>
+      </c>
       <c r="H11" s="2">
         <v>30</v>
       </c>
@@ -9958,6 +10044,12 @@
       </c>
       <c r="K11" t="s">
         <v>63</v>
+      </c>
+      <c r="L11" t="s">
+        <v>155</v>
+      </c>
+      <c r="M11" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9979,6 +10071,9 @@
       <c r="F12" s="2">
         <v>11</v>
       </c>
+      <c r="G12" t="s">
+        <v>155</v>
+      </c>
       <c r="H12" s="2">
         <v>25</v>
       </c>
@@ -9990,6 +10085,12 @@
       </c>
       <c r="K12" t="s">
         <v>63</v>
+      </c>
+      <c r="L12" t="s">
+        <v>155</v>
+      </c>
+      <c r="M12" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -10011,6 +10112,9 @@
       <c r="F13" s="2">
         <v>12</v>
       </c>
+      <c r="G13" t="s">
+        <v>155</v>
+      </c>
       <c r="H13" s="2">
         <v>20</v>
       </c>
@@ -10022,6 +10126,12 @@
       </c>
       <c r="K13" t="s">
         <v>63</v>
+      </c>
+      <c r="L13" t="s">
+        <v>155</v>
+      </c>
+      <c r="M13" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -10043,6 +10153,9 @@
       <c r="F14" s="2">
         <v>13</v>
       </c>
+      <c r="G14" t="s">
+        <v>155</v>
+      </c>
       <c r="H14" s="2">
         <v>25</v>
       </c>
@@ -10054,6 +10167,12 @@
       </c>
       <c r="K14" t="s">
         <v>78</v>
+      </c>
+      <c r="L14" t="s">
+        <v>155</v>
+      </c>
+      <c r="M14" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -10075,6 +10194,9 @@
       <c r="F15" s="2">
         <v>14</v>
       </c>
+      <c r="G15" t="s">
+        <v>155</v>
+      </c>
       <c r="H15" s="2">
         <v>20</v>
       </c>
@@ -10086,6 +10208,12 @@
       </c>
       <c r="K15" t="s">
         <v>78</v>
+      </c>
+      <c r="L15" t="s">
+        <v>155</v>
+      </c>
+      <c r="M15" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -10107,6 +10235,9 @@
       <c r="F16" s="2">
         <v>15</v>
       </c>
+      <c r="G16" t="s">
+        <v>155</v>
+      </c>
       <c r="H16" s="2">
         <v>30</v>
       </c>
@@ -10119,8 +10250,14 @@
       <c r="K16" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" t="s">
+        <v>155</v>
+      </c>
+      <c r="M16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>88</v>
       </c>
@@ -10139,6 +10276,9 @@
       <c r="F17" s="2">
         <v>16</v>
       </c>
+      <c r="G17" t="s">
+        <v>155</v>
+      </c>
       <c r="H17" s="2">
         <v>35</v>
       </c>
@@ -10151,8 +10291,14 @@
       <c r="K17" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L17" t="s">
+        <v>155</v>
+      </c>
+      <c r="M17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -10171,6 +10317,9 @@
       <c r="F18" s="2">
         <v>17</v>
       </c>
+      <c r="G18" t="s">
+        <v>155</v>
+      </c>
       <c r="H18" s="2">
         <v>25</v>
       </c>
@@ -10183,8 +10332,14 @@
       <c r="K18" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L18" t="s">
+        <v>155</v>
+      </c>
+      <c r="M18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>99</v>
       </c>
@@ -10203,6 +10358,9 @@
       <c r="F19" s="2">
         <v>18</v>
       </c>
+      <c r="G19" t="s">
+        <v>155</v>
+      </c>
       <c r="H19" s="2">
         <v>50</v>
       </c>
@@ -10215,8 +10373,14 @@
       <c r="K19" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" t="s">
+        <v>155</v>
+      </c>
+      <c r="M19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>104</v>
       </c>
@@ -10235,6 +10399,9 @@
       <c r="F20" s="2">
         <v>19</v>
       </c>
+      <c r="G20" t="s">
+        <v>155</v>
+      </c>
       <c r="H20" s="2">
         <v>40</v>
       </c>
@@ -10247,8 +10414,14 @@
       <c r="K20" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L20" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>110</v>
       </c>
@@ -10267,6 +10440,9 @@
       <c r="F21" s="2">
         <v>20</v>
       </c>
+      <c r="G21" t="s">
+        <v>155</v>
+      </c>
       <c r="H21" s="2">
         <v>50</v>
       </c>
@@ -10279,8 +10455,14 @@
       <c r="K21" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L21" t="s">
+        <v>155</v>
+      </c>
+      <c r="M21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>115</v>
       </c>
@@ -10299,6 +10481,9 @@
       <c r="F22" s="2">
         <v>21</v>
       </c>
+      <c r="G22" t="s">
+        <v>155</v>
+      </c>
       <c r="H22" s="2">
         <v>60</v>
       </c>
@@ -10311,8 +10496,14 @@
       <c r="K22" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L22" t="s">
+        <v>155</v>
+      </c>
+      <c r="M22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>120</v>
       </c>
@@ -10331,6 +10522,9 @@
       <c r="F23" s="2">
         <v>22</v>
       </c>
+      <c r="G23" t="s">
+        <v>155</v>
+      </c>
       <c r="H23" s="2">
         <v>35</v>
       </c>
@@ -10343,8 +10537,14 @@
       <c r="K23" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L23" t="s">
+        <v>155</v>
+      </c>
+      <c r="M23" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>126</v>
       </c>
@@ -10363,6 +10563,9 @@
       <c r="F24" s="2">
         <v>23</v>
       </c>
+      <c r="G24" t="s">
+        <v>155</v>
+      </c>
       <c r="H24" s="2">
         <v>15</v>
       </c>
@@ -10375,8 +10578,14 @@
       <c r="K24" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L24" t="s">
+        <v>155</v>
+      </c>
+      <c r="M24" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>131</v>
       </c>
@@ -10395,6 +10604,9 @@
       <c r="F25" s="2">
         <v>24</v>
       </c>
+      <c r="G25" t="s">
+        <v>155</v>
+      </c>
       <c r="H25" s="2">
         <v>20</v>
       </c>
@@ -10407,8 +10619,14 @@
       <c r="K25" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L25" t="s">
+        <v>155</v>
+      </c>
+      <c r="M25" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>136</v>
       </c>
@@ -10427,6 +10645,9 @@
       <c r="F26" s="2">
         <v>25</v>
       </c>
+      <c r="G26" t="s">
+        <v>155</v>
+      </c>
       <c r="H26" s="2">
         <v>40</v>
       </c>
@@ -10439,8 +10660,14 @@
       <c r="K26" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L26" t="s">
+        <v>155</v>
+      </c>
+      <c r="M26" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>142</v>
       </c>
@@ -10459,6 +10686,9 @@
       <c r="F27" s="2">
         <v>26</v>
       </c>
+      <c r="G27" t="s">
+        <v>155</v>
+      </c>
       <c r="H27" s="2">
         <v>25</v>
       </c>
@@ -10471,8 +10701,14 @@
       <c r="K27" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L27" t="s">
+        <v>155</v>
+      </c>
+      <c r="M27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>147</v>
       </c>
@@ -10491,6 +10727,9 @@
       <c r="F28" s="2">
         <v>27</v>
       </c>
+      <c r="G28" t="s">
+        <v>155</v>
+      </c>
       <c r="H28" s="2">
         <v>45</v>
       </c>
@@ -10502,6 +10741,12 @@
       </c>
       <c r="K28" t="s">
         <v>141</v>
+      </c>
+      <c r="L28" t="s">
+        <v>155</v>
+      </c>
+      <c r="M28" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -30171,7 +30416,9 @@
     <col min="6" max="6" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="139.33203125" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30234,6 +30481,9 @@
       <c r="F2" s="2">
         <v>1</v>
       </c>
+      <c r="G2" t="s">
+        <v>155</v>
+      </c>
       <c r="H2" s="2">
         <v>50</v>
       </c>
@@ -30245,6 +30495,12 @@
       </c>
       <c r="K2" t="s">
         <v>495</v>
+      </c>
+      <c r="L2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M2" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30266,6 +30522,9 @@
       <c r="F3" s="2">
         <v>2</v>
       </c>
+      <c r="G3" t="s">
+        <v>155</v>
+      </c>
       <c r="H3" s="2">
         <v>40</v>
       </c>
@@ -30277,6 +30536,12 @@
       </c>
       <c r="K3" t="s">
         <v>495</v>
+      </c>
+      <c r="L3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30298,6 +30563,9 @@
       <c r="F4" s="2">
         <v>3</v>
       </c>
+      <c r="G4" t="s">
+        <v>155</v>
+      </c>
       <c r="H4" s="2">
         <v>35</v>
       </c>
@@ -30309,6 +30577,12 @@
       </c>
       <c r="K4" t="s">
         <v>495</v>
+      </c>
+      <c r="L4" t="s">
+        <v>155</v>
+      </c>
+      <c r="M4" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30330,6 +30604,9 @@
       <c r="F5" s="2">
         <v>4</v>
       </c>
+      <c r="G5" t="s">
+        <v>155</v>
+      </c>
       <c r="H5" s="2">
         <v>45</v>
       </c>
@@ -30341,6 +30618,12 @@
       </c>
       <c r="K5" t="s">
         <v>495</v>
+      </c>
+      <c r="L5" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30362,6 +30645,9 @@
       <c r="F6" s="2">
         <v>5</v>
       </c>
+      <c r="G6" t="s">
+        <v>155</v>
+      </c>
       <c r="H6" s="2">
         <v>60</v>
       </c>
@@ -30373,6 +30659,12 @@
       </c>
       <c r="K6" t="s">
         <v>511</v>
+      </c>
+      <c r="L6" t="s">
+        <v>155</v>
+      </c>
+      <c r="M6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30394,6 +30686,9 @@
       <c r="F7" s="2">
         <v>6</v>
       </c>
+      <c r="G7" t="s">
+        <v>155</v>
+      </c>
       <c r="H7" s="2">
         <v>55</v>
       </c>
@@ -30405,6 +30700,12 @@
       </c>
       <c r="K7" t="s">
         <v>511</v>
+      </c>
+      <c r="L7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M7" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30426,6 +30727,9 @@
       <c r="F8" s="2">
         <v>7</v>
       </c>
+      <c r="G8" t="s">
+        <v>155</v>
+      </c>
       <c r="H8" s="2">
         <v>45</v>
       </c>
@@ -30437,6 +30741,12 @@
       </c>
       <c r="K8" t="s">
         <v>511</v>
+      </c>
+      <c r="L8" t="s">
+        <v>155</v>
+      </c>
+      <c r="M8" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30458,6 +30768,9 @@
       <c r="F9" s="2">
         <v>8</v>
       </c>
+      <c r="G9" t="s">
+        <v>155</v>
+      </c>
       <c r="H9" s="2">
         <v>50</v>
       </c>
@@ -30469,6 +30782,12 @@
       </c>
       <c r="K9" t="s">
         <v>511</v>
+      </c>
+      <c r="L9" t="s">
+        <v>155</v>
+      </c>
+      <c r="M9" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30490,6 +30809,9 @@
       <c r="F10" s="2">
         <v>9</v>
       </c>
+      <c r="G10" t="s">
+        <v>155</v>
+      </c>
       <c r="H10" s="2">
         <v>70</v>
       </c>
@@ -30501,6 +30823,12 @@
       </c>
       <c r="K10" t="s">
         <v>526</v>
+      </c>
+      <c r="L10" t="s">
+        <v>155</v>
+      </c>
+      <c r="M10" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30522,6 +30850,9 @@
       <c r="F11" s="2">
         <v>10</v>
       </c>
+      <c r="G11" t="s">
+        <v>155</v>
+      </c>
       <c r="H11" s="2">
         <v>65</v>
       </c>
@@ -30533,6 +30864,12 @@
       </c>
       <c r="K11" t="s">
         <v>526</v>
+      </c>
+      <c r="L11" t="s">
+        <v>155</v>
+      </c>
+      <c r="M11" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30554,6 +30891,9 @@
       <c r="F12" s="2">
         <v>11</v>
       </c>
+      <c r="G12" t="s">
+        <v>155</v>
+      </c>
       <c r="H12" s="2">
         <v>80</v>
       </c>
@@ -30565,6 +30905,12 @@
       </c>
       <c r="K12" t="s">
         <v>526</v>
+      </c>
+      <c r="L12" t="s">
+        <v>155</v>
+      </c>
+      <c r="M12" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30586,6 +30932,9 @@
       <c r="F13" s="2">
         <v>12</v>
       </c>
+      <c r="G13" t="s">
+        <v>155</v>
+      </c>
       <c r="H13" s="2">
         <v>60</v>
       </c>
@@ -30597,6 +30946,12 @@
       </c>
       <c r="K13" t="s">
         <v>526</v>
+      </c>
+      <c r="L13" t="s">
+        <v>155</v>
+      </c>
+      <c r="M13" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30618,6 +30973,9 @@
       <c r="F14" s="2">
         <v>13</v>
       </c>
+      <c r="G14" t="s">
+        <v>155</v>
+      </c>
       <c r="H14" s="2">
         <v>40</v>
       </c>
@@ -30629,6 +30987,12 @@
       </c>
       <c r="K14" t="s">
         <v>543</v>
+      </c>
+      <c r="L14" t="s">
+        <v>155</v>
+      </c>
+      <c r="M14" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30650,6 +31014,9 @@
       <c r="F15" s="2">
         <v>14</v>
       </c>
+      <c r="G15" t="s">
+        <v>155</v>
+      </c>
       <c r="H15" s="2">
         <v>55</v>
       </c>
@@ -30661,6 +31028,12 @@
       </c>
       <c r="K15" t="s">
         <v>543</v>
+      </c>
+      <c r="L15" t="s">
+        <v>155</v>
+      </c>
+      <c r="M15" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30682,6 +31055,9 @@
       <c r="F16" s="2">
         <v>15</v>
       </c>
+      <c r="G16" t="s">
+        <v>155</v>
+      </c>
       <c r="H16" s="2">
         <v>45</v>
       </c>
@@ -30694,8 +31070,14 @@
       <c r="K16" t="s">
         <v>543</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" t="s">
+        <v>155</v>
+      </c>
+      <c r="M16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>553</v>
       </c>
@@ -30714,6 +31096,9 @@
       <c r="F17" s="2">
         <v>16</v>
       </c>
+      <c r="G17" t="s">
+        <v>155</v>
+      </c>
       <c r="H17" s="2">
         <v>50</v>
       </c>
@@ -30726,8 +31111,14 @@
       <c r="K17" t="s">
         <v>543</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L17" t="s">
+        <v>155</v>
+      </c>
+      <c r="M17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>557</v>
       </c>
@@ -30746,6 +31137,9 @@
       <c r="F18" s="2">
         <v>17</v>
       </c>
+      <c r="G18" t="s">
+        <v>155</v>
+      </c>
       <c r="H18" s="2">
         <v>30</v>
       </c>
@@ -30758,8 +31152,14 @@
       <c r="K18" t="s">
         <v>561</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L18" t="s">
+        <v>155</v>
+      </c>
+      <c r="M18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>562</v>
       </c>
@@ -30778,6 +31178,9 @@
       <c r="F19" s="2">
         <v>18</v>
       </c>
+      <c r="G19" t="s">
+        <v>155</v>
+      </c>
       <c r="H19" s="2">
         <v>25</v>
       </c>
@@ -30790,8 +31193,14 @@
       <c r="K19" t="s">
         <v>561</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" t="s">
+        <v>155</v>
+      </c>
+      <c r="M19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>566</v>
       </c>
@@ -30810,6 +31219,9 @@
       <c r="F20" s="2">
         <v>19</v>
       </c>
+      <c r="G20" t="s">
+        <v>155</v>
+      </c>
       <c r="H20" s="2">
         <v>20</v>
       </c>
@@ -30822,8 +31234,14 @@
       <c r="K20" t="s">
         <v>561</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L20" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>570</v>
       </c>
@@ -30842,6 +31260,9 @@
       <c r="F21" s="2">
         <v>20</v>
       </c>
+      <c r="G21" t="s">
+        <v>155</v>
+      </c>
       <c r="H21" s="2">
         <v>28</v>
       </c>
@@ -30853,6 +31274,12 @@
       </c>
       <c r="K21" t="s">
         <v>561</v>
+      </c>
+      <c r="L21" t="s">
+        <v>155</v>
+      </c>
+      <c r="M21" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -30874,7 +31301,9 @@
     <col min="6" max="6" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="132.5" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30937,6 +31366,9 @@
       <c r="F2" s="2">
         <v>1</v>
       </c>
+      <c r="G2" t="s">
+        <v>155</v>
+      </c>
       <c r="H2" s="2">
         <v>100</v>
       </c>
@@ -30948,6 +31380,12 @@
       </c>
       <c r="K2" t="s">
         <v>454</v>
+      </c>
+      <c r="L2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M2" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -30969,6 +31407,9 @@
       <c r="F3" s="2">
         <v>2</v>
       </c>
+      <c r="G3" t="s">
+        <v>155</v>
+      </c>
       <c r="H3" s="2">
         <v>80</v>
       </c>
@@ -30980,6 +31421,12 @@
       </c>
       <c r="K3" t="s">
         <v>454</v>
+      </c>
+      <c r="L3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31001,6 +31448,9 @@
       <c r="F4" s="2">
         <v>3</v>
       </c>
+      <c r="G4" t="s">
+        <v>155</v>
+      </c>
       <c r="H4" s="2">
         <v>60</v>
       </c>
@@ -31012,6 +31462,12 @@
       </c>
       <c r="K4" t="s">
         <v>454</v>
+      </c>
+      <c r="L4" t="s">
+        <v>155</v>
+      </c>
+      <c r="M4" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31033,6 +31489,9 @@
       <c r="F5" s="2">
         <v>4</v>
       </c>
+      <c r="G5" t="s">
+        <v>155</v>
+      </c>
       <c r="H5" s="2">
         <v>50</v>
       </c>
@@ -31044,6 +31503,12 @@
       </c>
       <c r="K5" t="s">
         <v>454</v>
+      </c>
+      <c r="L5" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31065,6 +31530,9 @@
       <c r="F6" s="2">
         <v>5</v>
       </c>
+      <c r="G6" t="s">
+        <v>155</v>
+      </c>
       <c r="H6" s="2">
         <v>70</v>
       </c>
@@ -31076,6 +31544,12 @@
       </c>
       <c r="K6" t="s">
         <v>454</v>
+      </c>
+      <c r="L6" t="s">
+        <v>155</v>
+      </c>
+      <c r="M6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31097,6 +31571,9 @@
       <c r="F7" s="2">
         <v>6</v>
       </c>
+      <c r="G7" t="s">
+        <v>155</v>
+      </c>
       <c r="H7" s="2">
         <v>70</v>
       </c>
@@ -31108,6 +31585,12 @@
       </c>
       <c r="K7" t="s">
         <v>477</v>
+      </c>
+      <c r="L7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M7" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31129,6 +31612,9 @@
       <c r="F8" s="2">
         <v>7</v>
       </c>
+      <c r="G8" t="s">
+        <v>155</v>
+      </c>
       <c r="H8" s="2">
         <v>40</v>
       </c>
@@ -31140,6 +31626,12 @@
       </c>
       <c r="K8" t="s">
         <v>477</v>
+      </c>
+      <c r="L8" t="s">
+        <v>155</v>
+      </c>
+      <c r="M8" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31161,6 +31653,9 @@
       <c r="F9" s="2">
         <v>8</v>
       </c>
+      <c r="G9" t="s">
+        <v>155</v>
+      </c>
       <c r="H9" s="2">
         <v>35</v>
       </c>
@@ -31172,6 +31667,12 @@
       </c>
       <c r="K9" t="s">
         <v>477</v>
+      </c>
+      <c r="L9" t="s">
+        <v>155</v>
+      </c>
+      <c r="M9" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31193,6 +31694,9 @@
       <c r="F10" s="2">
         <v>9</v>
       </c>
+      <c r="G10" t="s">
+        <v>155</v>
+      </c>
       <c r="H10" s="2">
         <v>55</v>
       </c>
@@ -31204,6 +31708,12 @@
       </c>
       <c r="K10" t="s">
         <v>477</v>
+      </c>
+      <c r="L10" t="s">
+        <v>155</v>
+      </c>
+      <c r="M10" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -31226,7 +31736,9 @@
     <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="46.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="13" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="132" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31289,6 +31801,9 @@
       <c r="F2" s="2">
         <v>1</v>
       </c>
+      <c r="G2" t="s">
+        <v>155</v>
+      </c>
       <c r="H2" s="2">
         <v>60</v>
       </c>
@@ -31300,6 +31815,12 @@
       </c>
       <c r="K2" t="s">
         <v>350</v>
+      </c>
+      <c r="L2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M2" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31321,6 +31842,9 @@
       <c r="F3" s="2">
         <v>2</v>
       </c>
+      <c r="G3" t="s">
+        <v>155</v>
+      </c>
       <c r="H3" s="2">
         <v>50</v>
       </c>
@@ -31332,6 +31856,12 @@
       </c>
       <c r="K3" t="s">
         <v>350</v>
+      </c>
+      <c r="L3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31353,6 +31883,9 @@
       <c r="F4" s="2">
         <v>3</v>
       </c>
+      <c r="G4" t="s">
+        <v>155</v>
+      </c>
       <c r="H4" s="2">
         <v>80</v>
       </c>
@@ -31364,6 +31897,12 @@
       </c>
       <c r="K4" t="s">
         <v>350</v>
+      </c>
+      <c r="L4" t="s">
+        <v>155</v>
+      </c>
+      <c r="M4" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31385,6 +31924,9 @@
       <c r="F5" s="2">
         <v>4</v>
       </c>
+      <c r="G5" t="s">
+        <v>155</v>
+      </c>
       <c r="H5" s="2">
         <v>55</v>
       </c>
@@ -31396,6 +31938,12 @@
       </c>
       <c r="K5" t="s">
         <v>350</v>
+      </c>
+      <c r="L5" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31417,6 +31965,9 @@
       <c r="F6" s="2">
         <v>5</v>
       </c>
+      <c r="G6" t="s">
+        <v>155</v>
+      </c>
       <c r="H6" s="2">
         <v>70</v>
       </c>
@@ -31428,6 +31979,12 @@
       </c>
       <c r="K6" t="s">
         <v>369</v>
+      </c>
+      <c r="L6" t="s">
+        <v>155</v>
+      </c>
+      <c r="M6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31449,6 +32006,9 @@
       <c r="F7" s="2">
         <v>6</v>
       </c>
+      <c r="G7" t="s">
+        <v>155</v>
+      </c>
       <c r="H7" s="2">
         <v>55</v>
       </c>
@@ -31460,6 +32020,12 @@
       </c>
       <c r="K7" t="s">
         <v>369</v>
+      </c>
+      <c r="L7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M7" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31481,6 +32047,9 @@
       <c r="F8" s="2">
         <v>7</v>
       </c>
+      <c r="G8" t="s">
+        <v>155</v>
+      </c>
       <c r="H8" s="2">
         <v>45</v>
       </c>
@@ -31492,6 +32061,12 @@
       </c>
       <c r="K8" t="s">
         <v>369</v>
+      </c>
+      <c r="L8" t="s">
+        <v>155</v>
+      </c>
+      <c r="M8" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31513,6 +32088,9 @@
       <c r="F9" s="2">
         <v>8</v>
       </c>
+      <c r="G9" t="s">
+        <v>155</v>
+      </c>
       <c r="H9" s="2">
         <v>35</v>
       </c>
@@ -31524,6 +32102,12 @@
       </c>
       <c r="K9" t="s">
         <v>369</v>
+      </c>
+      <c r="L9" t="s">
+        <v>155</v>
+      </c>
+      <c r="M9" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31545,6 +32129,9 @@
       <c r="F10" s="2">
         <v>9</v>
       </c>
+      <c r="G10" t="s">
+        <v>155</v>
+      </c>
       <c r="H10" s="2">
         <v>90</v>
       </c>
@@ -31556,6 +32143,12 @@
       </c>
       <c r="K10" t="s">
         <v>389</v>
+      </c>
+      <c r="L10" t="s">
+        <v>155</v>
+      </c>
+      <c r="M10" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31577,6 +32170,9 @@
       <c r="F11" s="2">
         <v>10</v>
       </c>
+      <c r="G11" t="s">
+        <v>155</v>
+      </c>
       <c r="H11" s="2">
         <v>40</v>
       </c>
@@ -31588,6 +32184,12 @@
       </c>
       <c r="K11" t="s">
         <v>389</v>
+      </c>
+      <c r="L11" t="s">
+        <v>155</v>
+      </c>
+      <c r="M11" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31609,6 +32211,9 @@
       <c r="F12" s="2">
         <v>11</v>
       </c>
+      <c r="G12" t="s">
+        <v>155</v>
+      </c>
       <c r="H12" s="2">
         <v>55</v>
       </c>
@@ -31620,6 +32225,12 @@
       </c>
       <c r="K12" t="s">
         <v>389</v>
+      </c>
+      <c r="L12" t="s">
+        <v>155</v>
+      </c>
+      <c r="M12" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31641,6 +32252,9 @@
       <c r="F13" s="2">
         <v>12</v>
       </c>
+      <c r="G13" t="s">
+        <v>155</v>
+      </c>
       <c r="H13" s="2">
         <v>65</v>
       </c>
@@ -31652,6 +32266,12 @@
       </c>
       <c r="K13" t="s">
         <v>389</v>
+      </c>
+      <c r="L13" t="s">
+        <v>155</v>
+      </c>
+      <c r="M13" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31673,6 +32293,9 @@
       <c r="F14" s="2">
         <v>13</v>
       </c>
+      <c r="G14" t="s">
+        <v>155</v>
+      </c>
       <c r="H14" s="2">
         <v>65</v>
       </c>
@@ -31684,6 +32307,12 @@
       </c>
       <c r="K14" t="s">
         <v>410</v>
+      </c>
+      <c r="L14" t="s">
+        <v>155</v>
+      </c>
+      <c r="M14" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31705,6 +32334,9 @@
       <c r="F15" s="2">
         <v>14</v>
       </c>
+      <c r="G15" t="s">
+        <v>155</v>
+      </c>
       <c r="H15" s="2">
         <v>70</v>
       </c>
@@ -31716,6 +32348,12 @@
       </c>
       <c r="K15" t="s">
         <v>410</v>
+      </c>
+      <c r="L15" t="s">
+        <v>155</v>
+      </c>
+      <c r="M15" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -31737,6 +32375,9 @@
       <c r="F16" s="2">
         <v>15</v>
       </c>
+      <c r="G16" t="s">
+        <v>155</v>
+      </c>
       <c r="H16" s="2">
         <v>30</v>
       </c>
@@ -31749,8 +32390,14 @@
       <c r="K16" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" t="s">
+        <v>155</v>
+      </c>
+      <c r="M16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>420</v>
       </c>
@@ -31769,6 +32416,9 @@
       <c r="F17" s="2">
         <v>16</v>
       </c>
+      <c r="G17" t="s">
+        <v>155</v>
+      </c>
       <c r="H17" s="2">
         <v>80</v>
       </c>
@@ -31781,8 +32431,14 @@
       <c r="K17" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L17" t="s">
+        <v>155</v>
+      </c>
+      <c r="M17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>426</v>
       </c>
@@ -31801,6 +32457,9 @@
       <c r="F18" s="2">
         <v>17</v>
       </c>
+      <c r="G18" t="s">
+        <v>155</v>
+      </c>
       <c r="H18" s="2">
         <v>75</v>
       </c>
@@ -31813,8 +32472,14 @@
       <c r="K18" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L18" t="s">
+        <v>155</v>
+      </c>
+      <c r="M18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>430</v>
       </c>
@@ -31833,6 +32498,9 @@
       <c r="F19" s="2">
         <v>18</v>
       </c>
+      <c r="G19" t="s">
+        <v>155</v>
+      </c>
       <c r="H19" s="2">
         <v>55</v>
       </c>
@@ -31845,8 +32513,14 @@
       <c r="K19" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" t="s">
+        <v>155</v>
+      </c>
+      <c r="M19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>434</v>
       </c>
@@ -31865,6 +32539,9 @@
       <c r="F20" s="2">
         <v>19</v>
       </c>
+      <c r="G20" t="s">
+        <v>155</v>
+      </c>
       <c r="H20" s="2">
         <v>60</v>
       </c>
@@ -31877,8 +32554,14 @@
       <c r="K20" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L20" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>440</v>
       </c>
@@ -31897,6 +32580,9 @@
       <c r="F21" s="2">
         <v>20</v>
       </c>
+      <c r="G21" t="s">
+        <v>155</v>
+      </c>
       <c r="H21" s="2">
         <v>50</v>
       </c>
@@ -31909,8 +32595,14 @@
       <c r="K21" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L21" t="s">
+        <v>155</v>
+      </c>
+      <c r="M21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>444</v>
       </c>
@@ -31929,6 +32621,9 @@
       <c r="F22" s="2">
         <v>21</v>
       </c>
+      <c r="G22" t="s">
+        <v>155</v>
+      </c>
       <c r="H22" s="2">
         <v>45</v>
       </c>
@@ -31940,6 +32635,12 @@
       </c>
       <c r="K22" t="s">
         <v>439</v>
+      </c>
+      <c r="L22" t="s">
+        <v>155</v>
+      </c>
+      <c r="M22" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>